<commit_message>
premier essai gestion des doc word en 3 langues
</commit_message>
<xml_diff>
--- a/Data_communes/lib_familles_produits.xlsx
+++ b/Data_communes/lib_familles_produits.xlsx
@@ -2786,8 +2786,8 @@
   <dimension ref="A1:F1000"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="4"/>
-    <col min="2" max="2" width="34.7109375" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="50.28515625" customWidth="1"/>
     <col min="3" max="3" width="56.140625" customWidth="1"/>
     <col min="4" max="4" width="73.7109375" customWidth="1"/>
     <col min="5" max="5" width="35.28515625" customWidth="1"/>

</xml_diff>